<commit_message>
update msg and banner
</commit_message>
<xml_diff>
--- a/bots.xlsx
+++ b/bots.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sd/Documents/GitHub/MarketingTelegramBot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EED9B585-8C19-3242-9D6D-DDE2C042E10D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92D76C2B-35D0-FF49-8A35-24BDB11AF5D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="61">
   <si>
     <t>bot_token</t>
   </si>
@@ -52,15 +52,9 @@
     <t>BDG555</t>
   </si>
   <si>
-    <t>Welcome To BDG 555! Thanks for using this bot.</t>
-  </si>
-  <si>
     <t>welcome_image</t>
   </si>
   <si>
-    <t>https://placehold.net/400x400.png</t>
-  </si>
-  <si>
     <t>z</t>
   </si>
   <si>
@@ -152,9 +146,6 @@
   </si>
   <si>
     <t>8657805504:AAFC3U3bBS7wtRs9ulUfC_PJzNmQD7mlfVg</t>
-  </si>
-  <si>
-    <t>https://cdn.multibet27.com/91C/promotions/banner/deposit1.webp</t>
   </si>
   <si>
     <t>https://cdn.multibet27.com/91C/promotions/banner/lossback.webp</t>
@@ -172,6 +163,142 @@
 📌 Registration Link 🚀
 http://91kkr.com/
 ⚠️ 18+ Only | Gamble Responsibly</t>
+  </si>
+  <si>
+    <t>🎰 91cric – Your Winning Partner! 🔥
+🟢 Sign up now &amp; grab instant bonus 🎁
+💸 4X Deposit Offer: 50% → 80% → 100% → 120%
+🚀 Total 350% bonus boost
+📉 6 Days Loss Cover for safe play 🔄
+👥 Refer &amp; Earn unlimited 💰
+📌 Register Now: http://91kkr.com/
+⚠️ 18+ Only | Play Responsibly</t>
+  </si>
+  <si>
+    <t>🔥 Start Winning with 91cric 🎰
+🎁 Instant Signup Bonus Available
+💸 Deposit &amp; Get up to 350% Extra
+📉 6 Days Loss Recovery Offer
+👥 Invite Friends &amp; Earn Daily 💰
+🚀 Don’t miss the action
+📌 Join Now: http://91kkr.com/
+⚠️ 18+ Only</t>
+  </si>
+  <si>
+    <t>🎰 Welcome to 91cric 🔥
+🟢 Register &amp; unlock bonuses instantly 🎁
+💸 Get 4X Deposit Advantage
+🚀 Up to 350% Bonus
+📉 Safe Play with Loss Recovery
+👥 Earn with Referral Program 💰
+📌 Sign up: http://91kkr.com/</t>
+  </si>
+  <si>
+    <t>🔥 91cric – Bet Smart, Win Big 🎰
+🎁 Signup Bonus waiting for you
+💸 50% to 120% Deposit Boost
+🚀 Total 350% Benefit
+📉 6 Days Safety Net
+👥 Invite &amp; Earn 💰
+📌 Join today: http://91kkr.com/</t>
+  </si>
+  <si>
+    <t>🎰 Ready to Win with 91cric? 🔥
+🎁 Get instant joining bonus
+💸 Deposit Bonus up to 350%
+📉 Loss Recovery for 6 Days
+👥 Refer &amp; Earn Daily Income 💰
+📌 Register: http://91kkr.com/</t>
+  </si>
+  <si>
+    <t>🔥 Big Wins Start Here – 91cric 🎰
+🎁 Signup &amp; claim your bonus
+💸 4X Deposit Boost
+🚀 Up to 350% Extra
+📉 Play Safe with Loss Cover
+👥 Invite friends &amp; earn 💰
+📌 Join: http://91kkr.com/</t>
+  </si>
+  <si>
+    <t>🎰 91cric – Play. Earn. Repeat 🔥
+🎁 Instant Signup Bonus
+💸 Deposit &amp; get 350% Extra
+📉 6 Days Loss Recovery
+👥 Referral Income 💰
+📌 Start Now: http://91kkr.com/</t>
+  </si>
+  <si>
+    <t>🔥 Join 91cric Today 🎰
+🎁 Bonus on Signup
+💸 Huge Deposit Boost Offer
+🚀 Up to 350% Bonus
+📉 Risk-Free Play for 6 Days
+👥 Invite &amp; Earn 💰
+📌 Register: http://91kkr.com/</t>
+  </si>
+  <si>
+    <t>🎰 91cric – India’s Betting Hub 🔥
+🎁 Signup Bonus Live Now
+💸 4X Deposit Offer
+🚀 Total 350% Bonus
+📉 Loss Recovery Plan
+👥 Earn with referrals 💰
+📌 Join: http://91kkr.com/</t>
+  </si>
+  <si>
+    <t>🔥 91cric – Winning Made Easy 🎰
+🎁 Get instant bonus on signup
+💸 Deposit &amp; enjoy 350% boost
+📉 6 Days Loss Recovery
+👥 Refer &amp; earn daily 💰
+📌 Register Now: http://91kkr.com/</t>
+  </si>
+  <si>
+    <t>🎰 Experience 91cric 🔥
+🎁 Instant joining bonus
+💸 Deposit bonus up to 350%
+📉 Safe play guarantee
+👥 Invite friends &amp; earn 💰
+📌 Join: http://91kkr.com/</t>
+  </si>
+  <si>
+    <t>🔥 Bet Bigger with 91cric 🎰
+🎁 Signup bonus available
+💸 4X Deposit Boost
+🚀 Up to 350% Extra
+📉 Loss recovery for 6 days
+👥 Referral earning 💰
+📌 Start: http://91kkr.com/</t>
+  </si>
+  <si>
+    <t>🎰 91cric – Play Smart 🔥
+🎁 Signup &amp; earn bonus
+💸 Deposit boost up to 350%
+📉 6 Days Safety Offer
+👥 Invite &amp; earn 💰
+📌 Register: http://91kkr.com/</t>
+  </si>
+  <si>
+    <t>🎰 91cric – Nonstop Winning 🔥
+🎁 Signup bonus unlocked
+💸 Deposit &amp; get 350%
+📉 6 Days loss protection
+👥 Invite &amp; earn 💰
+📌 Join: http://91kkr.com/</t>
+  </si>
+  <si>
+    <t>🔥 Play. Earn. Repeat 🎰
+🎁 Signup Bonus Ready
+💸 Deposit &amp; get 350% Extra
+📉 Loss Recovery Available
+👥 Referral Income 💰
+📌 Join Now: http://91kkr.com/</t>
+  </si>
+  <si>
+    <t>https://cdn.multibet27.com/TGBOT/IPL-2026.jpg</t>
+  </si>
+  <si>
+    <t>https://cdn.multibet27.com/TGBOT/welcome-bonus.png</t>
   </si>
 </sst>
 </file>
@@ -586,7 +713,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -601,7 +728,7 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -621,10 +748,10 @@
         <v>7</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -637,19 +764,19 @@
       <c r="D3" t="s">
         <v>4</v>
       </c>
-      <c r="E3" t="s">
-        <v>10</v>
+      <c r="E3" s="3" t="s">
+        <v>44</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>12</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="360" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C4">
         <v>7375254799</v>
@@ -658,18 +785,18 @@
         <v>4</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="340" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C5">
         <v>7375254799</v>
@@ -678,18 +805,18 @@
         <v>4</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="340" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C6">
         <v>7375254799</v>
@@ -701,15 +828,15 @@
         <v>46</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="340" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C7">
         <v>7375254799</v>
@@ -718,18 +845,18 @@
         <v>4</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="340" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C8">
         <v>7375254799</v>
@@ -738,18 +865,18 @@
         <v>4</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="340" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C9">
         <v>7375254799</v>
@@ -758,18 +885,18 @@
         <v>4</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="340" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C10">
         <v>7375254799</v>
@@ -778,18 +905,18 @@
         <v>4</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="340" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C11">
         <v>7375254799</v>
@@ -798,18 +925,18 @@
         <v>4</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="340" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C12">
         <v>7375254799</v>
@@ -818,18 +945,18 @@
         <v>4</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="340" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C13">
         <v>7375254800</v>
@@ -838,18 +965,18 @@
         <v>4</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="340" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C14">
         <v>7375254801</v>
@@ -858,18 +985,18 @@
         <v>4</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="340" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C15">
         <v>7375254802</v>
@@ -878,18 +1005,18 @@
         <v>4</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="340" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C16">
         <v>7375254803</v>
@@ -898,18 +1025,18 @@
         <v>4</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="340" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C17">
         <v>7375254804</v>
@@ -918,18 +1045,18 @@
         <v>4</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="340" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C18">
         <v>7375254805</v>
@@ -938,19 +1065,18 @@
         <v>4</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F4" r:id="rId1" xr:uid="{DD19CD24-0A42-1646-B6CD-49EBB62D5021}"/>
-    <hyperlink ref="F5" r:id="rId2" xr:uid="{C4017207-4CAC-2E4F-A49E-68621EE8F63D}"/>
-    <hyperlink ref="F3" r:id="rId3" xr:uid="{AE2774FC-2067-074C-AA90-3A44A25D2846}"/>
-    <hyperlink ref="F2" r:id="rId4" xr:uid="{B5973262-4429-3E42-BB02-67D86243D83F}"/>
-    <hyperlink ref="F6:F18" r:id="rId5" display="https://cdn.multibet27.com/91C/promotions/banner/lossback.webp" xr:uid="{7F6EFC8D-5408-0B46-AFE2-FE88828B81A9}"/>
+    <hyperlink ref="F3" r:id="rId1" xr:uid="{AE2774FC-2067-074C-AA90-3A44A25D2846}"/>
+    <hyperlink ref="F2" r:id="rId2" xr:uid="{B5973262-4429-3E42-BB02-67D86243D83F}"/>
+    <hyperlink ref="F4:F18" r:id="rId3" display="https://cdn.multibet27.com/TGBOT/welcome-bonus.png" xr:uid="{2B19A97B-F01F-2345-8C23-D5420FEAD18C}"/>
+    <hyperlink ref="F17" r:id="rId4" xr:uid="{7AECAE2B-4790-104B-9926-25FDB5D1EB7F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>